<commit_message>
Populate protocol from DB: capture schedule №Протокол, replace hardcoded reviewer/grades with placeholders, add exam grade inputs
- loaders.py: detect unnamed column after «Дипломный руководитель» in schedule sheets and treat it as «Протокол» (fixes #57 missing)
- v1 template (data/протоколШАБЛОн.docx): replace hardcoded Батенина, Суворкина, 58 страниц, exam scores, ГИА grade with placeholders {Рецензент}, {Руководитель_исходный}, {ВКР}, {ГрафЧасть}, {БаллДемо}, {оценкаДемо}, {оценкаДиплом}, {ГИА}, {Дата_ДЭ}; remove duplicated paragraphs
- diploma.py / store.py: persist extra text fields (БаллДемо, оценкаДемо, оценкаДиплом, ГИА, Дата_ДЭ) as overrides
- diplomas.html / diploma.js: editable inputs for exam scores and ДЭ date
- data files: refresh with user-provided ДП/Защита versions

Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Form2Act-master/data/Защита по дням (ИС) (1) (1).xlsx
+++ b/Form2Act-master/data/Защита по дням (ИС) (1) (1).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\205\Desktop\Form2Act-master\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\205\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{457AE73C-4604-4CED-B360-CC8AA837F7E5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54F00A96-8FDF-41A5-89E7-C5C5B1EAA379}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23655" windowHeight="7965" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="16.06.25" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="128">
   <si>
     <t>№</t>
   </si>
@@ -41,6 +41,9 @@
     <t>Дипломный руководитель</t>
   </si>
   <si>
+    <t>Карпеев Арсений Алексеевич</t>
+  </si>
+  <si>
     <t>Кондратов Кирилл Алексеевич</t>
   </si>
   <si>
@@ -251,9 +254,6 @@
     <t>Тамбовцев Данила Александрович</t>
   </si>
   <si>
-    <t>Цапаев Александр Алексеевич</t>
-  </si>
-  <si>
     <t>23.06.2025 (ПОНЕДЕЛЬНИК)</t>
   </si>
   <si>
@@ -413,20 +413,14 @@
     <t>43ис</t>
   </si>
   <si>
-    <t>Протокол</t>
-  </si>
-  <si>
-    <t>Грибаков Андрей Сергеевич</t>
-  </si>
-  <si>
-    <t>Голубев Владимир Александрович</t>
+    <t>Шумейко Василий Александрович</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -478,14 +472,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
@@ -555,7 +541,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -591,16 +577,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -955,12 +932,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="A1" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
@@ -971,27 +948,25 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="18" t="s">
-        <v>127</v>
-      </c>
+      <c r="E2" s="6"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>129</v>
+        <v>3</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -1008,13 +983,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -1025,13 +1000,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -1045,13 +1020,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6">
         <v>4</v>
@@ -1065,13 +1040,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E7">
         <v>5</v>
@@ -1082,13 +1057,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E8">
         <v>6</v>
@@ -1102,13 +1077,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E9">
         <v>7</v>
@@ -1119,13 +1094,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E10">
         <v>8</v>
@@ -1139,13 +1114,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E11">
         <v>9</v>
@@ -1159,13 +1134,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E12">
         <v>10</v>
@@ -1173,32 +1148,32 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1223,12 +1198,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -1239,7 +1214,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
@@ -1325,7 +1300,7 @@
         <v>83</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E7" s="6">
         <v>113</v>
@@ -1342,7 +1317,7 @@
         <v>83</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E8" s="6">
         <v>114</v>
@@ -1359,7 +1334,7 @@
         <v>83</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E9" s="6">
         <v>115</v>
@@ -1376,7 +1351,7 @@
         <v>83</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E10" s="6">
         <v>116</v>
@@ -1400,32 +1375,32 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1452,7 +1427,7 @@
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C5">
         <v>27</v>
@@ -1506,12 +1481,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="A1" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
@@ -1522,7 +1497,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
@@ -1537,13 +1512,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3">
         <v>11</v>
@@ -1554,13 +1529,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4">
         <v>12</v>
@@ -1574,13 +1549,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E5">
         <v>13</v>
@@ -1594,13 +1569,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6">
         <v>14</v>
@@ -1611,13 +1586,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7">
         <v>15</v>
@@ -1631,13 +1606,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8">
         <v>16</v>
@@ -1648,13 +1623,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E9">
         <v>17</v>
@@ -1692,32 +1667,32 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1742,12 +1717,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="A1" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
@@ -1758,7 +1733,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
@@ -1770,13 +1745,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E3">
         <v>18</v>
@@ -1787,13 +1762,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4">
         <v>19</v>
@@ -1804,13 +1779,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E5">
         <v>20</v>
@@ -1821,13 +1796,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6">
         <v>21</v>
@@ -1838,13 +1813,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7">
         <v>22</v>
@@ -1855,13 +1830,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E8">
         <v>23</v>
@@ -1872,13 +1847,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9">
         <v>24</v>
@@ -1889,13 +1864,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E10">
         <v>25</v>
@@ -1906,13 +1881,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E11">
         <v>26</v>
@@ -1926,13 +1901,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E12">
         <v>27</v>
@@ -1940,32 +1915,32 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1991,12 +1966,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="A1" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2007,7 +1982,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
@@ -2019,13 +1994,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3">
         <v>28</v>
@@ -2036,13 +2011,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E4">
         <v>29</v>
@@ -2053,13 +2028,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E5">
         <v>30</v>
@@ -2070,13 +2045,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E6">
         <v>31</v>
@@ -2087,13 +2062,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7">
         <v>32</v>
@@ -2104,13 +2079,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E8">
         <v>33</v>
@@ -2121,13 +2096,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9">
         <v>34</v>
@@ -2138,13 +2113,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E10">
         <v>35</v>
@@ -2155,13 +2130,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11">
         <v>36</v>
@@ -2172,13 +2147,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E12">
         <v>37</v>
@@ -2189,13 +2164,13 @@
         <v>11</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E13">
         <v>38</v>
@@ -2206,13 +2181,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E14">
         <v>39</v>
@@ -2229,32 +2204,32 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -2268,7 +2243,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.28515625" customWidth="1"/>
@@ -2279,89 +2254,79 @@
     <col min="9" max="9" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="10"/>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="15" t="s">
+      <c r="C2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
-        <v>1</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="E2">
-        <v>51</v>
-      </c>
+      <c r="E2" s="6"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>68</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E3">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>69</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="E4">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>70</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="D5" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E5">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
         <v>115</v>
@@ -2369,120 +2334,134 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>71</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>47</v>
+        <v>66</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="E6">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>72</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>13</v>
+        <v>66</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="E7">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>73</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="D8" s="2" t="s">
         <v>66</v>
       </c>
+      <c r="D8" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="E8">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>47</v>
+        <v>7</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="E9">
-        <f>E8+11</f>
-        <v>68</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="8"/>
       <c r="D10" s="4"/>
+      <c r="E10">
+        <f>E9+11</f>
+        <v>68</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="8"/>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="9" t="s">
-        <v>23</v>
-      </c>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="2"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>14</v>
+      <c r="B16" s="9" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="9" t="s">
-        <v>49</v>
+      <c r="B17" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
+      <c r="B18" s="9" t="s">
         <v>50</v>
       </c>
     </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -2502,12 +2481,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="A1" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
@@ -2518,7 +2497,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
@@ -2535,7 +2514,7 @@
       <c r="C3" s="8"/>
       <c r="D3" s="4"/>
       <c r="E3">
-        <f>'20.06.25'!E9+14</f>
+        <f>'20.06.25'!E10+14</f>
         <v>82</v>
       </c>
     </row>
@@ -2557,23 +2536,23 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10"/>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
@@ -2582,7 +2561,7 @@
     <row r="11" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11"/>
       <c r="B11" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
@@ -2591,7 +2570,7 @@
     <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12"/>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
@@ -2619,12 +2598,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2635,7 +2614,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
@@ -2650,13 +2629,13 @@
         <v>79</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3" s="6">
-        <f>14+'20.06.25'!E9+1</f>
+        <f>14+'20.06.25'!E10+1</f>
         <v>83</v>
       </c>
     </row>
@@ -2668,10 +2647,10 @@
         <v>80</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E4" s="6">
         <v>84</v>
@@ -2685,10 +2664,10 @@
         <v>75</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E5" s="6">
         <v>85</v>
@@ -2702,10 +2681,10 @@
         <v>76</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E6" s="6">
         <v>86</v>
@@ -2719,10 +2698,10 @@
         <v>77</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E7" s="6">
         <v>87</v>
@@ -2736,10 +2715,10 @@
         <v>78</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8" s="6">
         <v>88</v>
@@ -2753,10 +2732,10 @@
         <v>81</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="6">
         <v>89</v>
@@ -2770,10 +2749,10 @@
         <v>112</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E10" s="6">
         <v>90</v>
@@ -2797,32 +2776,32 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -2847,12 +2826,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -2863,7 +2842,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
@@ -2881,7 +2860,7 @@
         <v>83</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" s="6">
         <v>91</v>
@@ -2898,7 +2877,7 @@
         <v>83</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E4" s="6">
         <v>92</v>
@@ -2915,7 +2894,7 @@
         <v>83</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E5" s="6">
         <v>93</v>
@@ -2932,7 +2911,7 @@
         <v>83</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E6" s="6">
         <v>94</v>
@@ -2949,7 +2928,7 @@
         <v>83</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E7" s="6">
         <v>95</v>
@@ -2966,7 +2945,7 @@
         <v>83</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E8" s="6">
         <v>96</v>
@@ -2983,7 +2962,7 @@
         <v>83</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E9" s="6">
         <v>97</v>
@@ -3000,7 +2979,7 @@
         <v>83</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E10" s="6">
         <v>98</v>
@@ -3017,7 +2996,7 @@
         <v>83</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" s="6">
         <v>99</v>
@@ -3033,32 +3012,32 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -3083,12 +3062,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="10"/>
     </row>
     <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
@@ -3099,7 +3078,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
@@ -3117,7 +3096,7 @@
         <v>83</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E3" s="6">
         <v>100</v>
@@ -3134,7 +3113,7 @@
         <v>83</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E4" s="6">
         <v>101</v>
@@ -3168,7 +3147,7 @@
         <v>83</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E6" s="6">
         <v>103</v>
@@ -3185,7 +3164,7 @@
         <v>83</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E7" s="6">
         <v>104</v>
@@ -3219,7 +3198,7 @@
         <v>83</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E9" s="6">
         <v>106</v>
@@ -3236,7 +3215,7 @@
         <v>83</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E10" s="6">
         <v>107</v>
@@ -3253,7 +3232,7 @@
         <v>83</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E11" s="6">
         <v>108</v>
@@ -3269,32 +3248,32 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>